<commit_message>
Actualizacion desde ordenador local: cambios en app.py, calculos_pilares.py, estilos y plantillas
</commit_message>
<xml_diff>
--- a/uploads/Excel_Ejemplo_Ratios_Financieros.xlsx
+++ b/uploads/Excel_Ejemplo_Ratios_Financieros.xlsx
@@ -1,22 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marpa\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69C557FE-3CFF-4897-A05C-CBCA677F4C68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98DC4453-BB79-4412-80CE-1329E204A5B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Balance_y_PyG" sheetId="1" r:id="rId1"/>
     <sheet name="LEEME" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -215,7 +226,7 @@
     <t xml:space="preserve">   para que reconozca tus conceptos específicos</t>
   </si>
   <si>
-    <t>BN</t>
+    <t>Resultado del ejercicio</t>
   </si>
 </sst>
 </file>
@@ -251,8 +262,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -556,12 +568,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F44"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -581,12 +593,12 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -606,7 +618,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -626,7 +638,7 @@
         <v>18000</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -646,7 +658,7 @@
         <v>42000</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -666,7 +678,7 @@
         <v>132000</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -686,7 +698,7 @@
         <v>39600</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -706,7 +718,7 @@
         <v>66000</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -726,7 +738,7 @@
         <v>26400</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -746,12 +758,12 @@
         <v>192000</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -771,7 +783,7 @@
         <v>99200</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -791,7 +803,7 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -811,7 +823,7 @@
         <v>37200</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>14</v>
       </c>
@@ -831,7 +843,7 @@
         <v>34800</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -851,7 +863,7 @@
         <v>34800</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -871,7 +883,7 @@
         <v>52800</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>17</v>
       </c>
@@ -891,7 +903,7 @@
         <v>15840</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>18</v>
       </c>
@@ -911,7 +923,7 @@
         <v>26400</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>19</v>
       </c>
@@ -931,7 +943,7 @@
         <v>10560</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>20</v>
       </c>
@@ -951,7 +963,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>21</v>
       </c>
@@ -971,7 +983,7 @@
         <v>280000</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>22</v>
       </c>
@@ -991,7 +1003,7 @@
         <v>280000</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -1011,7 +1023,7 @@
         <v>81599.999999999985</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>24</v>
       </c>
@@ -1031,7 +1043,7 @@
         <v>196000</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>25</v>
       </c>
@@ -1051,7 +1063,7 @@
         <v>47520</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>26</v>
       </c>
@@ -1071,7 +1083,7 @@
         <v>151360</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>27</v>
       </c>
@@ -1091,7 +1103,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>28</v>
       </c>
@@ -1111,7 +1123,7 @@
         <v>-2357</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>29</v>
       </c>
@@ -1131,7 +1143,7 @@
         <v>-1143</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>30</v>
       </c>
@@ -1151,7 +1163,7 @@
         <v>148963</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>31</v>
       </c>
@@ -1171,14 +1183,14 @@
         <v>-37240.75</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>64</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="1">
         <v>77323.5</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="1">
         <v>85212.000000000029</v>
       </c>
       <c r="D39">
@@ -1191,7 +1203,7 @@
         <v>111722.25</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>32</v>
       </c>
@@ -1211,7 +1223,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>33</v>
       </c>
@@ -1231,7 +1243,7 @@
         <v>46148</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>34</v>
       </c>
@@ -1251,7 +1263,7 @@
         <v>9137</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>35</v>
       </c>
@@ -1279,144 +1291,144 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>63</v>
       </c>

</xml_diff>

<commit_message>
Renombra acronimo BETTY, unifica bandas de interpretacion con el Glosario y agrega documentos de TFM
</commit_message>
<xml_diff>
--- a/uploads/Excel_Ejemplo_Ratios_Financieros.xlsx
+++ b/uploads/Excel_Ejemplo_Ratios_Financieros.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marpa\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98DC4453-BB79-4412-80CE-1329E204A5B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B200D49E-DDC0-4630-8F7E-12A7E345DB3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,18 +16,7 @@
     <sheet name="Balance_y_PyG" sheetId="1" r:id="rId1"/>
     <sheet name="LEEME" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 

</xml_diff>